<commit_message>
split ldpe and mldpe.
</commit_message>
<xml_diff>
--- a/outputs/optionen-v2-2026-09-29/Optionen-Vergleich-v2.xlsx
+++ b/outputs/optionen-v2-2026-09-29/Optionen-Vergleich-v2.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beispielpositionen" sheetId="1" r:id="Re8921990bcd64f91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feldmapping" sheetId="2" r:id="R73704cf797e042e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beispielpositionen" sheetId="1" r:id="Re61f86c7b0934d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feldmapping" sheetId="2" r:id="R586c70f09fe24736"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,9 +14,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="0.000"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.000"/>
+    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="203" formatCode="#,##0.###"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="205" formatCode="dd.mm.yyyy"/>
+    <x:numFmt numFmtId="206" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -82,7 +87,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -102,6 +107,46 @@
     <x:xf numFmtId="201" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -330,6 +375,9 @@
     <x:col min="20" max="20" width="78" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="28" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="28" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="42" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="72" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -360,7 +408,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>DB04/BMS, live gelesen am 29.09.2026. Testgültigkeit bis 27.10.2026. Leere kg- und €/t-Felder bedeuten: Einheit nicht bestätigt.</x:v>
+        <x:v>Live-Abgleich DB04/BMS vom 02.10.2026: 11 Angebote (7 Demo, 4 echte Eingänge), 16 Positionen. Einheiten bleiben unbestätigt, wenn kg- bzw. Preiseinheit/€/t in der Quelle nicht belegt sind.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -451,482 +499,959 @@
       <x:c r="V5" s="6" t="str">
         <x:v>Quelldatei</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="46" customHeight="1">
-      <x:c r="A6" s="7" t="str">
+      <x:c r="W5" s="29" t="str">
+        <x:v>Artikelindex-Vorschlag</x:v>
+      </x:c>
+      <x:c r="X5" s="29" t="str">
+        <x:v>Wahrscheinlicher Artikel bei uns</x:v>
+      </x:c>
+      <x:c r="Y5" s="29" t="str">
+        <x:v>Begründung des App-Vorschlags</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="18" t="str">
         <x:v>TotalEnergies</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
+      <x:c r="B6" s="18" t="str">
         <x:v>2037660</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="str">
-        <x:v>2026-09-06</x:v>
-      </x:c>
-      <x:c r="D6" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="str">
+      <x:c r="C6" s="27" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D6" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E6" s="18" t="str">
         <x:v>PPH 10000 OG</x:v>
       </x:c>
-      <x:c r="F6" s="7" t="str">
+      <x:c r="F6" s="18" t="str">
         <x:v>6G04DBA0</x:v>
       </x:c>
-      <x:c r="G6" s="7" t="str">
+      <x:c r="G6" s="18" t="str">
         <x:v>PP Homo</x:v>
       </x:c>
-      <x:c r="H6" s="7" t="str">
+      <x:c r="H6" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I6" s="8" t="n">
+      <x:c r="I6" s="20" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="J6" s="7"/>
-      <x:c r="K6" s="8"/>
-      <x:c r="L6" s="7"/>
-      <x:c r="M6" s="10" t="str">
+      <x:c r="J6" s="18"/>
+      <x:c r="K6" s="20"/>
+      <x:c r="L6" s="18"/>
+      <x:c r="M6" s="21" t="str">
         <x:v>2.750 (XFA-Wert; Einheit nicht angegeben)</x:v>
       </x:c>
-      <x:c r="N6" s="7"/>
-      <x:c r="O6" s="9"/>
-      <x:c r="P6" s="9"/>
-      <x:c r="Q6" s="11" t="n">
+      <x:c r="N6" s="18"/>
+      <x:c r="O6" s="22"/>
+      <x:c r="P6" s="22"/>
+      <x:c r="Q6" s="23" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="R6" s="9"/>
-      <x:c r="S6" s="12"/>
-      <x:c r="T6" s="13" t="str">
-        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet.</x:v>
-      </x:c>
-      <x:c r="U6" s="7" t="str">
+      <x:c r="R6" s="24"/>
+      <x:c r="S6" s="25"/>
+      <x:c r="T6" s="26" t="str">
+        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: BAGS Incoterm: FCA Ladeort: PP Feluy</x:v>
+      </x:c>
+      <x:c r="U6" s="18" t="str">
         <x:v>suggested</x:v>
       </x:c>
-      <x:c r="V6" s="7" t="str">
+      <x:c r="V6" s="18" t="str">
         <x:v>Offer  2037660.PDF</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="46" customHeight="1">
-      <x:c r="A7" s="7" t="str">
+      <x:c r="W6" s="28" t="str">
+        <x:v>02213</x:v>
+      </x:c>
+      <x:c r="X6" s="18" t="str">
+        <x:v>PP Homo NT MFI 40-50 natur</x:v>
+      </x:c>
+      <x:c r="Y6" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 40–50. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="18" t="str">
         <x:v>TotalEnergies</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="str">
+      <x:c r="B7" s="18" t="str">
         <x:v>2037660</x:v>
       </x:c>
-      <x:c r="C7" s="7" t="str">
-        <x:v>2026-09-06</x:v>
-      </x:c>
-      <x:c r="D7" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="str">
+      <x:c r="C7" s="27" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D7" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E7" s="18" t="str">
         <x:v>PPH 10000 OG</x:v>
       </x:c>
-      <x:c r="F7" s="7" t="str">
+      <x:c r="F7" s="18" t="str">
         <x:v>6H13DBD3</x:v>
       </x:c>
-      <x:c r="G7" s="7" t="str">
+      <x:c r="G7" s="18" t="str">
         <x:v>PP Homo</x:v>
       </x:c>
-      <x:c r="H7" s="7" t="str">
+      <x:c r="H7" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I7" s="8" t="n">
+      <x:c r="I7" s="20" t="n">
         <x:v>36.7</x:v>
       </x:c>
-      <x:c r="J7" s="7"/>
-      <x:c r="K7" s="8"/>
-      <x:c r="L7" s="7"/>
-      <x:c r="M7" s="10" t="str">
+      <x:c r="J7" s="18"/>
+      <x:c r="K7" s="20"/>
+      <x:c r="L7" s="18"/>
+      <x:c r="M7" s="21" t="str">
         <x:v>19.250 (XFA-Wert; Einheit nicht angegeben)</x:v>
       </x:c>
-      <x:c r="N7" s="7"/>
-      <x:c r="O7" s="9"/>
-      <x:c r="P7" s="9"/>
-      <x:c r="Q7" s="11" t="n">
+      <x:c r="N7" s="18"/>
+      <x:c r="O7" s="22"/>
+      <x:c r="P7" s="22"/>
+      <x:c r="Q7" s="23" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="R7" s="9"/>
-      <x:c r="S7" s="12"/>
-      <x:c r="T7" s="13" t="str">
-        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet.</x:v>
-      </x:c>
-      <x:c r="U7" s="7" t="str">
+      <x:c r="R7" s="24"/>
+      <x:c r="S7" s="25"/>
+      <x:c r="T7" s="26" t="str">
+        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: BAGS Incoterm: FCA Ladeort: PP Feluy</x:v>
+      </x:c>
+      <x:c r="U7" s="18" t="str">
         <x:v>suggested</x:v>
       </x:c>
-      <x:c r="V7" s="7" t="str">
+      <x:c r="V7" s="18" t="str">
         <x:v>Offer  2037660.PDF</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="46" customHeight="1">
-      <x:c r="A8" s="7" t="str">
+      <x:c r="W7" s="28" t="str">
+        <x:v>02212</x:v>
+      </x:c>
+      <x:c r="X7" s="18" t="str">
+        <x:v>PP Homo NT MFI 30-40 natur</x:v>
+      </x:c>
+      <x:c r="Y7" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 30–40. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="18" t="str">
         <x:v>TotalEnergies</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="str">
+      <x:c r="B8" s="18" t="str">
         <x:v>2037688</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="D8" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E8" s="7" t="str">
+      <x:c r="C8" s="27" t="d">
+        <x:v>2026-09-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E8" s="18" t="str">
         <x:v>PPH 10000 OG</x:v>
       </x:c>
-      <x:c r="F8" s="7" t="str">
+      <x:c r="F8" s="18" t="str">
         <x:v>6H05DBB2</x:v>
       </x:c>
-      <x:c r="G8" s="7" t="str">
+      <x:c r="G8" s="18" t="str">
         <x:v>PP Homo</x:v>
       </x:c>
-      <x:c r="H8" s="7" t="str">
+      <x:c r="H8" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I8" s="8" t="n">
+      <x:c r="I8" s="20" t="n">
         <x:v>35.7</x:v>
       </x:c>
-      <x:c r="J8" s="7"/>
-      <x:c r="K8" s="8"/>
-      <x:c r="L8" s="7"/>
-      <x:c r="M8" s="10" t="str">
+      <x:c r="J8" s="18"/>
+      <x:c r="K8" s="20"/>
+      <x:c r="L8" s="18"/>
+      <x:c r="M8" s="21" t="str">
         <x:v>99.000 (XFA-Wert; Einheit nicht angegeben)</x:v>
       </x:c>
-      <x:c r="N8" s="7"/>
-      <x:c r="O8" s="9"/>
-      <x:c r="P8" s="9"/>
-      <x:c r="Q8" s="11" t="n">
+      <x:c r="N8" s="18"/>
+      <x:c r="O8" s="22"/>
+      <x:c r="P8" s="22"/>
+      <x:c r="Q8" s="23" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="R8" s="9"/>
-      <x:c r="S8" s="12"/>
-      <x:c r="T8" s="13" t="str">
-        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet.</x:v>
-      </x:c>
-      <x:c r="U8" s="7" t="str">
+      <x:c r="R8" s="24"/>
+      <x:c r="S8" s="25"/>
+      <x:c r="T8" s="26" t="str">
+        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: BAGS Incoterm: FCA Ladeort: PP Feluy</x:v>
+      </x:c>
+      <x:c r="U8" s="18" t="str">
         <x:v>suggested</x:v>
       </x:c>
-      <x:c r="V8" s="7" t="str">
+      <x:c r="V8" s="18" t="str">
         <x:v>Offer  2037688.PDF</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="46" customHeight="1">
-      <x:c r="A9" s="7" t="str">
+      <x:c r="W8" s="28" t="str">
+        <x:v>02212</x:v>
+      </x:c>
+      <x:c r="X8" s="18" t="str">
+        <x:v>PP Homo NT MFI 30-40 natur</x:v>
+      </x:c>
+      <x:c r="Y8" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 30–40. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="18" t="str">
         <x:v>TotalEnergies</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="str">
+      <x:c r="B9" s="18" t="str">
         <x:v>2037746</x:v>
       </x:c>
-      <x:c r="C9" s="7" t="str">
-        <x:v>2026-09-14</x:v>
-      </x:c>
-      <x:c r="D9" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E9" s="7" t="str">
+      <x:c r="C9" s="27" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E9" s="18" t="str">
         <x:v>PEHD 2007TN61 near prime</x:v>
       </x:c>
-      <x:c r="F9" s="7" t="str">
+      <x:c r="F9" s="18" t="str">
         <x:v>P608033</x:v>
       </x:c>
-      <x:c r="G9" s="7" t="str">
+      <x:c r="G9" s="18" t="str">
         <x:v>HDPE</x:v>
       </x:c>
-      <x:c r="H9" s="7" t="str">
+      <x:c r="H9" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I9" s="8" t="n">
+      <x:c r="I9" s="20" t="n">
         <x:v>43.3</x:v>
       </x:c>
-      <x:c r="J9" s="7" t="str">
+      <x:c r="J9" s="18" t="str">
         <x:v>21.6 kg</x:v>
       </x:c>
-      <x:c r="K9" s="8" t="n">
+      <x:c r="K9" s="20" t="n">
         <x:v>959.1</x:v>
       </x:c>
-      <x:c r="L9" s="7"/>
-      <x:c r="M9" s="10" t="str">
+      <x:c r="L9" s="18"/>
+      <x:c r="M9" s="21" t="str">
         <x:v>156.750 (XFA-Wert; Einheit nicht angegeben)</x:v>
       </x:c>
-      <x:c r="N9" s="7"/>
-      <x:c r="O9" s="9"/>
-      <x:c r="P9" s="9"/>
-      <x:c r="Q9" s="11" t="n">
+      <x:c r="N9" s="18"/>
+      <x:c r="O9" s="22"/>
+      <x:c r="P9" s="22"/>
+      <x:c r="Q9" s="23" t="n">
         <x:v>970</x:v>
       </x:c>
-      <x:c r="R9" s="9"/>
-      <x:c r="S9" s="12"/>
-      <x:c r="T9" s="13" t="str">
-        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet.</x:v>
-      </x:c>
-      <x:c r="U9" s="7" t="str">
+      <x:c r="R9" s="24"/>
+      <x:c r="S9" s="25"/>
+      <x:c r="T9" s="26" t="str">
+        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: BAGS Incoterm: FCA Ladeort: Usine de Gonfreville L'Orcher</x:v>
+      </x:c>
+      <x:c r="U9" s="18" t="str">
         <x:v>suggested</x:v>
       </x:c>
-      <x:c r="V9" s="7" t="str">
+      <x:c r="V9" s="18" t="str">
         <x:v>Offer  2037746.PDF</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="46" customHeight="1">
-      <x:c r="A10" s="7" t="str">
+      <x:c r="W9" s="28" t="str">
+        <x:v>04757</x:v>
+      </x:c>
+      <x:c r="X9" s="18" t="str">
+        <x:v>HDPE NT MFI 40-49,99 (bei 21,6kg) natur</x:v>
+      </x:c>
+      <x:c r="Y9" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 40–49.99, MFI-Prüflast passt. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="56" customHeight="1">
+      <x:c r="A10" s="18" t="str">
         <x:v>TotalEnergies</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="str">
+      <x:c r="B10" s="18" t="str">
         <x:v>2037748</x:v>
       </x:c>
-      <x:c r="C10" s="7" t="str">
-        <x:v>2026-09-14</x:v>
-      </x:c>
-      <x:c r="D10" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E10" s="7" t="str">
+      <x:c r="C10" s="27" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D10" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E10" s="18" t="str">
         <x:v>PEHD 2008DN60 OG</x:v>
       </x:c>
-      <x:c r="F10" s="7" t="str">
+      <x:c r="F10" s="18" t="str">
         <x:v>P608038</x:v>
       </x:c>
-      <x:c r="G10" s="7" t="str">
+      <x:c r="G10" s="18" t="str">
         <x:v>HDPE</x:v>
       </x:c>
-      <x:c r="H10" s="7" t="str">
+      <x:c r="H10" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I10" s="8" t="n">
+      <x:c r="I10" s="20" t="n">
         <x:v>48.5</x:v>
       </x:c>
-      <x:c r="J10" s="7" t="str">
+      <x:c r="J10" s="18" t="str">
         <x:v>21.6 kg</x:v>
       </x:c>
-      <x:c r="K10" s="8" t="n">
+      <x:c r="K10" s="20" t="n">
         <x:v>959.2</x:v>
       </x:c>
-      <x:c r="L10" s="7"/>
-      <x:c r="M10" s="10" t="str">
+      <x:c r="L10" s="18"/>
+      <x:c r="M10" s="21" t="str">
         <x:v>47.400 (XFA-Wert; Einheit nicht angegeben)</x:v>
       </x:c>
-      <x:c r="N10" s="7"/>
-      <x:c r="O10" s="9"/>
-      <x:c r="P10" s="9"/>
-      <x:c r="Q10" s="11" t="n">
+      <x:c r="N10" s="18"/>
+      <x:c r="O10" s="22"/>
+      <x:c r="P10" s="22"/>
+      <x:c r="Q10" s="23" t="n">
         <x:v>950</x:v>
       </x:c>
-      <x:c r="R10" s="9"/>
-      <x:c r="S10" s="12"/>
-      <x:c r="T10" s="13" t="str">
-        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet.</x:v>
-      </x:c>
-      <x:c r="U10" s="7" t="str">
+      <x:c r="R10" s="24"/>
+      <x:c r="S10" s="25"/>
+      <x:c r="T10" s="26" t="str">
+        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: BAGS Incoterm: FCA Ladeort: Usine de Gonfreville L'Orcher</x:v>
+      </x:c>
+      <x:c r="U10" s="18" t="str">
         <x:v>suggested</x:v>
       </x:c>
-      <x:c r="V10" s="7" t="str">
+      <x:c r="V10" s="18" t="str">
         <x:v>Offer  2037748.PDF</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="46" customHeight="1">
-      <x:c r="A11" s="7" t="str">
+      <x:c r="W10" s="28" t="str">
+        <x:v>04757</x:v>
+      </x:c>
+      <x:c r="X10" s="18" t="str">
+        <x:v>HDPE NT MFI 40-49,99 (bei 21,6kg) natur</x:v>
+      </x:c>
+      <x:c r="Y10" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 40–49.99, MFI-Prüflast passt. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="56" customHeight="1">
+      <x:c r="A11" s="18" t="str">
         <x:v>TotalEnergies</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="str">
+      <x:c r="B11" s="18" t="str">
         <x:v>2037758</x:v>
       </x:c>
-      <x:c r="C11" s="7" t="str">
-        <x:v>2026-09-15</x:v>
-      </x:c>
-      <x:c r="D11" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E11" s="7" t="str">
+      <x:c r="C11" s="27" t="d">
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E11" s="18" t="str">
         <x:v>PPC 7600 OG</x:v>
       </x:c>
-      <x:c r="F11" s="7" t="str">
+      <x:c r="F11" s="18" t="str">
         <x:v>6G03DZB8</x:v>
       </x:c>
-      <x:c r="G11" s="7" t="str">
+      <x:c r="G11" s="18" t="str">
         <x:v>PP Copo</x:v>
       </x:c>
-      <x:c r="H11" s="7" t="str">
+      <x:c r="H11" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I11" s="8" t="n">
+      <x:c r="I11" s="20" t="n">
         <x:v>9.4</x:v>
       </x:c>
-      <x:c r="J11" s="7"/>
-      <x:c r="K11" s="8"/>
-      <x:c r="L11" s="7"/>
-      <x:c r="M11" s="10" t="str">
+      <x:c r="J11" s="18"/>
+      <x:c r="K11" s="20"/>
+      <x:c r="L11" s="18"/>
+      <x:c r="M11" s="21" t="str">
         <x:v>24.750 (XFA-Wert; Einheit nicht angegeben)</x:v>
       </x:c>
-      <x:c r="N11" s="7"/>
-      <x:c r="O11" s="9"/>
-      <x:c r="P11" s="9"/>
-      <x:c r="Q11" s="11" t="n">
+      <x:c r="N11" s="18"/>
+      <x:c r="O11" s="22"/>
+      <x:c r="P11" s="22"/>
+      <x:c r="Q11" s="23" t="n">
         <x:v>1030</x:v>
       </x:c>
-      <x:c r="R11" s="9"/>
-      <x:c r="S11" s="12"/>
-      <x:c r="T11" s="13" t="str">
-        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet.</x:v>
-      </x:c>
-      <x:c r="U11" s="7" t="str">
+      <x:c r="R11" s="24"/>
+      <x:c r="S11" s="25"/>
+      <x:c r="T11" s="26" t="str">
+        <x:v>Mengeneinheit nicht bestätigt; Rohmenge anzeigen. Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: BAGS Incoterm: FCA Ladeort: PP Feluy</x:v>
+      </x:c>
+      <x:c r="U11" s="18" t="str">
         <x:v>suggested</x:v>
       </x:c>
-      <x:c r="V11" s="7" t="str">
+      <x:c r="V11" s="18" t="str">
         <x:v>Offer  2037758.PDF</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="46" customHeight="1">
-      <x:c r="A12" s="7" t="str">
+      <x:c r="W11" s="28" t="str">
+        <x:v>04521</x:v>
+      </x:c>
+      <x:c r="X11" s="18" t="str">
+        <x:v>PP Copo NT MFI 8 - 9,9 natur</x:v>
+      </x:c>
+      <x:c r="Y11" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 8–9.9. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="56" customHeight="1">
+      <x:c r="A12" s="18" t="str">
         <x:v>Longfield Polymers</x:v>
       </x:c>
-      <x:c r="B12" s="7"/>
-      <x:c r="C12" s="7"/>
-      <x:c r="D12" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E12" s="7" t="str">
+      <x:c r="B12" s="18"/>
+      <x:c r="C12" s="27"/>
+      <x:c r="D12" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E12" s="18" t="str">
         <x:v>LDPE mfi 2.0 no adds near to prime</x:v>
       </x:c>
-      <x:c r="F12" s="7"/>
-      <x:c r="G12" s="7" t="str">
+      <x:c r="F12" s="18"/>
+      <x:c r="G12" s="18" t="str">
         <x:v>LDPE</x:v>
       </x:c>
-      <x:c r="H12" s="7" t="str">
+      <x:c r="H12" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I12" s="8" t="n">
+      <x:c r="I12" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="J12" s="7"/>
-      <x:c r="K12" s="8"/>
-      <x:c r="L12" s="7"/>
-      <x:c r="M12" s="10" t="str">
+      <x:c r="J12" s="18"/>
+      <x:c r="K12" s="20"/>
+      <x:c r="L12" s="18"/>
+      <x:c r="M12" s="21" t="str">
         <x:v>3 truckloads</x:v>
       </x:c>
-      <x:c r="N12" s="7" t="str">
+      <x:c r="N12" s="18" t="str">
         <x:v>truckload</x:v>
       </x:c>
-      <x:c r="O12" s="9"/>
-      <x:c r="P12" s="9"/>
-      <x:c r="Q12" s="11" t="n">
+      <x:c r="O12" s="22"/>
+      <x:c r="P12" s="22"/>
+      <x:c r="Q12" s="23" t="n">
         <x:v>1150</x:v>
       </x:c>
-      <x:c r="R12" s="9" t="str">
+      <x:c r="R12" s="24" t="str">
         <x:v>EUR/t</x:v>
       </x:c>
-      <x:c r="S12" s="12" t="n">
+      <x:c r="S12" s="25" t="n">
         <x:v>1150</x:v>
       </x:c>
-      <x:c r="T12" s="13" t="str">
-        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg.</x:v>
-      </x:c>
-      <x:c r="U12" s="7" t="str">
+      <x:c r="T12" s="26" t="str">
+        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg. Packed 25kg bags on pallets; loading prompt after order or 1st October Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: 25 kg bags Incoterm: FCA Ladeort: Holland</x:v>
+      </x:c>
+      <x:c r="U12" s="18" t="str">
         <x:v>unmatched</x:v>
       </x:c>
-      <x:c r="V12" s="7" t="str">
+      <x:c r="V12" s="18" t="str">
         <x:v>codex-clipboard-6d92da5b-8835-4a05-8444-2d304b9508b0.png</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="46" customHeight="1">
-      <x:c r="A13" s="7" t="str">
+      <x:c r="W12" s="28"/>
+      <x:c r="X12" s="18"/>
+      <x:c r="Y12" s="26"/>
+    </x:row>
+    <x:row r="13" ht="56" customHeight="1">
+      <x:c r="A13" s="18" t="str">
         <x:v>Longfield Polymers</x:v>
       </x:c>
-      <x:c r="B13" s="7"/>
-      <x:c r="C13" s="7"/>
-      <x:c r="D13" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="str">
+      <x:c r="B13" s="18"/>
+      <x:c r="C13" s="27"/>
+      <x:c r="D13" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E13" s="18" t="str">
         <x:v>LDPE mfi 4.0 no adds near to prime</x:v>
       </x:c>
-      <x:c r="F13" s="7"/>
-      <x:c r="G13" s="7" t="str">
+      <x:c r="F13" s="18"/>
+      <x:c r="G13" s="18" t="str">
         <x:v>LDPE</x:v>
       </x:c>
-      <x:c r="H13" s="7" t="str">
+      <x:c r="H13" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I13" s="8" t="n">
+      <x:c r="I13" s="20" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="J13" s="7"/>
-      <x:c r="K13" s="8"/>
-      <x:c r="L13" s="7"/>
-      <x:c r="M13" s="10" t="str">
+      <x:c r="J13" s="18"/>
+      <x:c r="K13" s="20"/>
+      <x:c r="L13" s="18"/>
+      <x:c r="M13" s="21" t="str">
         <x:v>1 truckload</x:v>
       </x:c>
-      <x:c r="N13" s="7" t="str">
+      <x:c r="N13" s="18" t="str">
         <x:v>truckload</x:v>
       </x:c>
-      <x:c r="O13" s="9"/>
-      <x:c r="P13" s="9"/>
-      <x:c r="Q13" s="11" t="n">
+      <x:c r="O13" s="22"/>
+      <x:c r="P13" s="22"/>
+      <x:c r="Q13" s="23" t="n">
         <x:v>1150</x:v>
       </x:c>
-      <x:c r="R13" s="9" t="str">
+      <x:c r="R13" s="24" t="str">
         <x:v>EUR/t</x:v>
       </x:c>
-      <x:c r="S13" s="12" t="n">
+      <x:c r="S13" s="25" t="n">
         <x:v>1150</x:v>
       </x:c>
-      <x:c r="T13" s="13" t="str">
-        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg.</x:v>
-      </x:c>
-      <x:c r="U13" s="7" t="str">
+      <x:c r="T13" s="26" t="str">
+        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg. Packed 25kg bags on pallets; loading prompt after order or 1st October Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: 25 kg bags Incoterm: FCA Ladeort: Holland</x:v>
+      </x:c>
+      <x:c r="U13" s="18" t="str">
         <x:v>unmatched</x:v>
       </x:c>
-      <x:c r="V13" s="7" t="str">
+      <x:c r="V13" s="18" t="str">
         <x:v>codex-clipboard-6d92da5b-8835-4a05-8444-2d304b9508b0.png</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="46" customHeight="1">
-      <x:c r="A14" s="7" t="str">
+      <x:c r="W13" s="28"/>
+      <x:c r="X13" s="18"/>
+      <x:c r="Y13" s="26"/>
+    </x:row>
+    <x:row r="14" ht="56" customHeight="1">
+      <x:c r="A14" s="18" t="str">
         <x:v>Longfield Polymers</x:v>
       </x:c>
-      <x:c r="B14" s="7"/>
-      <x:c r="C14" s="7"/>
-      <x:c r="D14" s="7" t="str">
-        <x:v>2026-10-27</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="str">
+      <x:c r="B14" s="18"/>
+      <x:c r="C14" s="27"/>
+      <x:c r="D14" s="27" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E14" s="18" t="str">
         <x:v>PPHP mfi 12.0 near to prime</x:v>
       </x:c>
-      <x:c r="F14" s="7"/>
-      <x:c r="G14" s="7" t="str">
+      <x:c r="F14" s="18"/>
+      <x:c r="G14" s="18" t="str">
         <x:v>PP Homo</x:v>
       </x:c>
-      <x:c r="H14" s="7" t="str">
+      <x:c r="H14" s="18" t="str">
         <x:v>NT</x:v>
       </x:c>
-      <x:c r="I14" s="8" t="n">
+      <x:c r="I14" s="20" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J14" s="7"/>
-      <x:c r="K14" s="8"/>
-      <x:c r="L14" s="7"/>
-      <x:c r="M14" s="10" t="str">
+      <x:c r="J14" s="18"/>
+      <x:c r="K14" s="20"/>
+      <x:c r="L14" s="18"/>
+      <x:c r="M14" s="21" t="str">
         <x:v>1-2 truckloads</x:v>
       </x:c>
-      <x:c r="N14" s="7" t="str">
+      <x:c r="N14" s="18" t="str">
         <x:v>truckload</x:v>
       </x:c>
-      <x:c r="O14" s="9"/>
-      <x:c r="P14" s="9"/>
-      <x:c r="Q14" s="11" t="n">
+      <x:c r="O14" s="22"/>
+      <x:c r="P14" s="22"/>
+      <x:c r="Q14" s="23" t="n">
         <x:v>995</x:v>
       </x:c>
-      <x:c r="R14" s="9" t="str">
+      <x:c r="R14" s="24" t="str">
         <x:v>EUR/t</x:v>
       </x:c>
-      <x:c r="S14" s="12" t="n">
+      <x:c r="S14" s="25" t="n">
         <x:v>995</x:v>
       </x:c>
-      <x:c r="T14" s="13" t="str">
-        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg.</x:v>
-      </x:c>
-      <x:c r="U14" s="7" t="str">
+      <x:c r="T14" s="26" t="str">
+        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg. 25kg bags; loading prompt after order Beispielimport: Gültigkeit bis 27.10.2026 nur für App-Tests simuliert; ursprüngliche Frist separat gespeichert. Verpackung: 25 kg bags Incoterm: FCA Ladeort: Germany</x:v>
+      </x:c>
+      <x:c r="U14" s="18" t="str">
         <x:v>suggested</x:v>
       </x:c>
-      <x:c r="V14" s="7" t="str">
+      <x:c r="V14" s="18" t="str">
         <x:v>codex-clipboard-35fbdecd-e9be-46c1-96a4-fbeae40d6b5d.png</x:v>
       </x:c>
+      <x:c r="W14" s="28" t="str">
+        <x:v>02210</x:v>
+      </x:c>
+      <x:c r="X14" s="18" t="str">
+        <x:v>PP Homo NT MFI 10 - 14,9 natur</x:v>
+      </x:c>
+      <x:c r="Y14" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 10–14.9. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="56" customHeight="1">
+      <x:c r="A15" s="18" t="str">
+        <x:v>INEOS Olefins &amp; Polymers Europe</x:v>
+      </x:c>
+      <x:c r="B15" s="18" t="str">
+        <x:v>OG-34-429320.2-MXG</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D15" s="27" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E15" s="18" t="str">
+        <x:v>mLLDPE OG</x:v>
+      </x:c>
+      <x:c r="F15" s="18" t="str">
+        <x:v>L1700A</x:v>
+      </x:c>
+      <x:c r="G15" s="18"/>
+      <x:c r="H15" s="18" t="str">
+        <x:v>NT</x:v>
+      </x:c>
+      <x:c r="I15" s="20" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="J15" s="18"/>
+      <x:c r="K15" s="20" t="n">
+        <x:v>912.5</x:v>
+      </x:c>
+      <x:c r="L15" s="18"/>
+      <x:c r="M15" s="21" t="str">
+        <x:v>22,000</x:v>
+      </x:c>
+      <x:c r="N15" s="18" t="str">
+        <x:v>kg</x:v>
+      </x:c>
+      <x:c r="O15" s="22" t="n">
+        <x:v>22000</x:v>
+      </x:c>
+      <x:c r="P15" s="22" t="n">
+        <x:v>22000</x:v>
+      </x:c>
+      <x:c r="Q15" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R15" s="24"/>
+      <x:c r="S15" s="25"/>
+      <x:c r="T15" s="26" t="str">
+        <x:v>Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Produced at Cologne. Material has to be collected within 10 working days or latest before end of month. Die Angebotsgültigkeit ist abgelaufen. Der angegebene Preis beträgt 0,00 EUR; eine Preiseinheit ist nicht angegeben. 10 days due net.…</x:v>
+      </x:c>
+      <x:c r="U15" s="18" t="str">
+        <x:v>unmatched</x:v>
+      </x:c>
+      <x:c r="V15" s="18" t="str">
+        <x:v>OG-34-429320.2-MXG.pdf</x:v>
+      </x:c>
+      <x:c r="W15" s="28"/>
+      <x:c r="X15" s="18"/>
+      <x:c r="Y15" s="26"/>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="18" t="str">
+        <x:v>Longfield Chemicals Limited</x:v>
+      </x:c>
+      <x:c r="B16" s="18"/>
+      <x:c r="C16" s="27"/>
+      <x:c r="D16" s="27" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E16" s="18" t="str">
+        <x:v>LDPE mfi 20,0</x:v>
+      </x:c>
+      <x:c r="F16" s="18"/>
+      <x:c r="G16" s="18" t="str">
+        <x:v>LDPE</x:v>
+      </x:c>
+      <x:c r="H16" s="18" t="str">
+        <x:v>NT</x:v>
+      </x:c>
+      <x:c r="I16" s="20" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J16" s="18"/>
+      <x:c r="K16" s="20"/>
+      <x:c r="L16" s="18"/>
+      <x:c r="M16" s="21" t="str">
+        <x:v>1 truckload</x:v>
+      </x:c>
+      <x:c r="N16" s="18" t="str">
+        <x:v>truckload</x:v>
+      </x:c>
+      <x:c r="O16" s="22"/>
+      <x:c r="P16" s="22"/>
+      <x:c r="Q16" s="23" t="n">
+        <x:v>1250</x:v>
+      </x:c>
+      <x:c r="R16" s="24" t="str">
+        <x:v>EUR/t</x:v>
+      </x:c>
+      <x:c r="S16" s="25" t="n">
+        <x:v>1250</x:v>
+      </x:c>
+      <x:c r="T16" s="26" t="str">
+        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg. Loading prompt after order Incoterm: FCA Ladeort: Holland</x:v>
+      </x:c>
+      <x:c r="U16" s="18" t="str">
+        <x:v>unmatched</x:v>
+      </x:c>
+      <x:c r="V16" s="18" t="str">
+        <x:v>E-Mail-Text</x:v>
+      </x:c>
+      <x:c r="W16" s="28"/>
+      <x:c r="X16" s="18"/>
+      <x:c r="Y16" s="26"/>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="18" t="str">
+        <x:v>Longfield Chemicals Limited</x:v>
+      </x:c>
+      <x:c r="B17" s="18"/>
+      <x:c r="C17" s="27"/>
+      <x:c r="D17" s="27" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E17" s="18" t="str">
+        <x:v>LDPE mfi 15,0</x:v>
+      </x:c>
+      <x:c r="F17" s="18"/>
+      <x:c r="G17" s="18" t="str">
+        <x:v>LDPE</x:v>
+      </x:c>
+      <x:c r="H17" s="18" t="str">
+        <x:v>NT</x:v>
+      </x:c>
+      <x:c r="I17" s="20" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="J17" s="18"/>
+      <x:c r="K17" s="20"/>
+      <x:c r="L17" s="18"/>
+      <x:c r="M17" s="21" t="str">
+        <x:v>1 truckload</x:v>
+      </x:c>
+      <x:c r="N17" s="18" t="str">
+        <x:v>truckload</x:v>
+      </x:c>
+      <x:c r="O17" s="22"/>
+      <x:c r="P17" s="22"/>
+      <x:c r="Q17" s="23" t="n">
+        <x:v>1245</x:v>
+      </x:c>
+      <x:c r="R17" s="24" t="str">
+        <x:v>EUR/t</x:v>
+      </x:c>
+      <x:c r="S17" s="25" t="n">
+        <x:v>1245</x:v>
+      </x:c>
+      <x:c r="T17" s="26" t="str">
+        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg. Loading prompt after order Incoterm: FCA Ladeort: Holland</x:v>
+      </x:c>
+      <x:c r="U17" s="18" t="str">
+        <x:v>unmatched</x:v>
+      </x:c>
+      <x:c r="V17" s="18" t="str">
+        <x:v>E-Mail-Text</x:v>
+      </x:c>
+      <x:c r="W17" s="28"/>
+      <x:c r="X17" s="18"/>
+      <x:c r="Y17" s="26"/>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="18" t="str">
+        <x:v>Longfield Chemicals Limited</x:v>
+      </x:c>
+      <x:c r="B18" s="18"/>
+      <x:c r="C18" s="27"/>
+      <x:c r="D18" s="27" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E18" s="18" t="str">
+        <x:v>LDPE mfi 12,0</x:v>
+      </x:c>
+      <x:c r="F18" s="18"/>
+      <x:c r="G18" s="18" t="str">
+        <x:v>LDPE</x:v>
+      </x:c>
+      <x:c r="H18" s="18" t="str">
+        <x:v>NT</x:v>
+      </x:c>
+      <x:c r="I18" s="20" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J18" s="18"/>
+      <x:c r="K18" s="20"/>
+      <x:c r="L18" s="18"/>
+      <x:c r="M18" s="21" t="str">
+        <x:v>1 truckload</x:v>
+      </x:c>
+      <x:c r="N18" s="18" t="str">
+        <x:v>truckload</x:v>
+      </x:c>
+      <x:c r="O18" s="22"/>
+      <x:c r="P18" s="22"/>
+      <x:c r="Q18" s="23" t="n">
+        <x:v>1240</x:v>
+      </x:c>
+      <x:c r="R18" s="24" t="str">
+        <x:v>EUR/t</x:v>
+      </x:c>
+      <x:c r="S18" s="25" t="n">
+        <x:v>1240</x:v>
+      </x:c>
+      <x:c r="T18" s="26" t="str">
+        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg. Loading prompt after order Incoterm: FCA Ladeort: Holland</x:v>
+      </x:c>
+      <x:c r="U18" s="18" t="str">
+        <x:v>unmatched</x:v>
+      </x:c>
+      <x:c r="V18" s="18" t="str">
+        <x:v>E-Mail-Text</x:v>
+      </x:c>
+      <x:c r="W18" s="28"/>
+      <x:c r="X18" s="18"/>
+      <x:c r="Y18" s="26"/>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="18" t="str">
+        <x:v>Longfield Chemicals Limited</x:v>
+      </x:c>
+      <x:c r="B19" s="18"/>
+      <x:c r="C19" s="27"/>
+      <x:c r="D19" s="27" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E19" s="18" t="str">
+        <x:v>PPHP</x:v>
+      </x:c>
+      <x:c r="F19" s="18"/>
+      <x:c r="G19" s="18"/>
+      <x:c r="H19" s="18" t="str">
+        <x:v>NT</x:v>
+      </x:c>
+      <x:c r="I19" s="20" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J19" s="18"/>
+      <x:c r="K19" s="20"/>
+      <x:c r="L19" s="18"/>
+      <x:c r="M19" s="21" t="str">
+        <x:v>1-2 truckloads</x:v>
+      </x:c>
+      <x:c r="N19" s="18" t="str">
+        <x:v>truckload</x:v>
+      </x:c>
+      <x:c r="O19" s="22"/>
+      <x:c r="P19" s="22"/>
+      <x:c r="Q19" s="23" t="n">
+        <x:v>1085</x:v>
+      </x:c>
+      <x:c r="R19" s="24" t="str">
+        <x:v>EUR/t</x:v>
+      </x:c>
+      <x:c r="S19" s="25" t="n">
+        <x:v>1085</x:v>
+      </x:c>
+      <x:c r="T19" s="26" t="str">
+        <x:v>LKW-Menge ohne bestätigtes Ladegewicht; keine Umrechnung in kg. Collections prompt after order Incoterm: FCA Ladeort: Holland</x:v>
+      </x:c>
+      <x:c r="U19" s="18" t="str">
+        <x:v>suggested</x:v>
+      </x:c>
+      <x:c r="V19" s="18" t="str">
+        <x:v>E-Mail-Text</x:v>
+      </x:c>
+      <x:c r="W19" s="28" t="str">
+        <x:v>02210</x:v>
+      </x:c>
+      <x:c r="X19" s="18" t="str">
+        <x:v>PP Homo NT MFI 10 - 14,9 natur</x:v>
+      </x:c>
+      <x:c r="Y19" s="26" t="str">
+        <x:v>Eindeutiger MFI-/Typ-Treffer: Kunststofftyp passt, NT passt, MFI 10–14.9. Bitte bestätigen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="18" t="str">
+        <x:v>Holland Trading House Chemicals b.v.</x:v>
+      </x:c>
+      <x:c r="B20" s="18"/>
+      <x:c r="C20" s="27"/>
+      <x:c r="D20" s="27" t="d">
+        <x:v>2026-10-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E20" s="18" t="str">
+        <x:v>LDPE Lupolen 2221D</x:v>
+      </x:c>
+      <x:c r="F20" s="18"/>
+      <x:c r="G20" s="18" t="str">
+        <x:v>LDPE</x:v>
+      </x:c>
+      <x:c r="H20" s="18" t="str">
+        <x:v>1A</x:v>
+      </x:c>
+      <x:c r="I20" s="20" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="J20" s="18"/>
+      <x:c r="K20" s="20" t="n">
+        <x:v>0.922</x:v>
+      </x:c>
+      <x:c r="L20" s="18"/>
+      <x:c r="M20" s="21" t="str">
+        <x:v>46750 kg</x:v>
+      </x:c>
+      <x:c r="N20" s="18" t="str">
+        <x:v>kg</x:v>
+      </x:c>
+      <x:c r="O20" s="22" t="n">
+        <x:v>46750</x:v>
+      </x:c>
+      <x:c r="P20" s="22" t="n">
+        <x:v>46750</x:v>
+      </x:c>
+      <x:c r="Q20" s="23" t="n">
+        <x:v>1325</x:v>
+      </x:c>
+      <x:c r="R20" s="24"/>
+      <x:c r="S20" s="25"/>
+      <x:c r="T20" s="26" t="str">
+        <x:v>Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Preiseinheit nicht angegeben. Dichte ohne Einheit angegeben. Verpackung: 25 kg original bags on pallets of 1375 kg Incoterm: FCA Ladeort: Antwerp</x:v>
+      </x:c>
+      <x:c r="U20" s="18" t="str">
+        <x:v>unmatched</x:v>
+      </x:c>
+      <x:c r="V20" s="18" t="str">
+        <x:v>E-Mail-Text</x:v>
+      </x:c>
+      <x:c r="W20" s="28"/>
+      <x:c r="X20" s="18"/>
+      <x:c r="Y20" s="26"/>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="18" t="str">
+        <x:v>Holland Trading House Chemicals b.v.</x:v>
+      </x:c>
+      <x:c r="B21" s="18"/>
+      <x:c r="C21" s="27"/>
+      <x:c r="D21" s="27" t="d">
+        <x:v>2026-10-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E21" s="18" t="str">
+        <x:v>LDPE Lupolen 2221F</x:v>
+      </x:c>
+      <x:c r="F21" s="18"/>
+      <x:c r="G21" s="18" t="str">
+        <x:v>LDPE</x:v>
+      </x:c>
+      <x:c r="H21" s="18" t="str">
+        <x:v>1A</x:v>
+      </x:c>
+      <x:c r="I21" s="20" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="J21" s="18"/>
+      <x:c r="K21" s="20" t="n">
+        <x:v>0.922</x:v>
+      </x:c>
+      <x:c r="L21" s="18"/>
+      <x:c r="M21" s="21" t="str">
+        <x:v>23375 kg</x:v>
+      </x:c>
+      <x:c r="N21" s="18" t="str">
+        <x:v>kg</x:v>
+      </x:c>
+      <x:c r="O21" s="22" t="n">
+        <x:v>23375</x:v>
+      </x:c>
+      <x:c r="P21" s="22" t="n">
+        <x:v>23375</x:v>
+      </x:c>
+      <x:c r="Q21" s="23" t="n">
+        <x:v>1325</x:v>
+      </x:c>
+      <x:c r="R21" s="24"/>
+      <x:c r="S21" s="25"/>
+      <x:c r="T21" s="26" t="str">
+        <x:v>Preiseinheit nicht angegeben; kein Preis pro Tonne berechnet. Preiseinheit nicht angegeben. Dichte ohne Einheit angegeben. Verpackung: 25 kg original bags on pallets of 1375 kg Incoterm: FCA Ladeort: Antwerp</x:v>
+      </x:c>
+      <x:c r="U21" s="18" t="str">
+        <x:v>unmatched</x:v>
+      </x:c>
+      <x:c r="V21" s="18" t="str">
+        <x:v>E-Mail-Text</x:v>
+      </x:c>
+      <x:c r="W21" s="28"/>
+      <x:c r="X21" s="18"/>
+      <x:c r="Y21" s="26"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>